<commit_message>
feat: SEMANA09 tasas reales de AFP y fuentes
</commit_message>
<xml_diff>
--- a/Semana 09/Boleta_Pago.xlsx
+++ b/Semana 09/Boleta_Pago.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="150">
   <si>
     <t xml:space="preserve">Parámetros de la boleta de pago</t>
   </si>
@@ -121,7 +121,25 @@
     <t xml:space="preserve">Valores de prueba de la guía (solo casos de prueba)</t>
   </si>
   <si>
-    <t xml:space="preserve">Filas amarillas: para agregar las AFP reales con los valores publicados por la SBS (anota la fuente y la fecha). Aún no se han llenado.</t>
+    <t xml:space="preserve">Habitat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SBS: comisión sobre flujo y prima de seguro, devengue oct-2026. Leído en Buk y TrámitesPerú; falta confirmar en la tabla de la SBS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">26/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profuturo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Las 4 AFP reales usan comisión sobre flujo (porcentaje del sueldo). La comisión mixta (sobre saldo) no está modelada. Para el caso propio usa una AFP real; los casos 1 a 4 usan AFP Ejemplo, como pide la guía.</t>
   </si>
   <si>
     <t xml:space="preserve">Boleta de ejemplo</t>
@@ -623,7 +641,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -672,14 +690,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -689,6 +699,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1187,41 +1201,89 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12"/>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12"/>
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12"/>
-      <c r="B22" s="13"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="13"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
+    <row r="19" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>0.0147</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>0.0137</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <v>0.0155</v>
+      </c>
+      <c r="D20" s="7" t="n">
+        <v>0.0137</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>0.0137</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B22" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>0.0169</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>0.0137</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14" t="s">
-        <v>32</v>
+      <c r="A23" s="12" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1249,108 +1311,108 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="15" t="n">
+        <v>42</v>
+      </c>
+      <c r="B5" s="13" t="n">
         <v>3000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B6" s="16" t="n">
+        <v>43</v>
+      </c>
+      <c r="B6" s="14" t="n">
         <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>39</v>
+        <v>44</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="15" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B9" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="15" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="B10" s="17" t="n">
+        <v>48</v>
+      </c>
+      <c r="B10" s="16" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B11" s="17" t="n">
+        <v>49</v>
+      </c>
+      <c r="B11" s="16" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B12" s="15" t="n">
+        <v>50</v>
+      </c>
+      <c r="B12" s="13" t="n">
         <v>200</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B16" s="18" t="n">
+        <v>54</v>
+      </c>
+      <c r="B16" s="17" t="n">
         <f aca="false">B5/Parámetros!B12/Parámetros!B13</f>
         <v>12.5</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">ROUND(B5/Parámetros!B12*B6,2)</f>
@@ -1359,7 +1421,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="B18" s="8" t="n">
         <f aca="false">IF(B7="Sí",ROUND(Parámetros!B7,2),0)</f>
@@ -1368,7 +1430,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">ROUND(B16*(1+Parámetros!B10)*B10,2)</f>
@@ -1377,7 +1439,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">ROUND(B16*(1+Parámetros!B11)*B11,2)</f>
@@ -1385,25 +1447,25 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="B21" s="20" t="n">
+      <c r="A21" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="B21" s="19" t="n">
         <f aca="false">SUM(B17:B20)</f>
         <v>3253</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B24" s="8" t="n">
         <f aca="false">IF(B8="ONP",ROUND(B21*Parámetros!B8,2),0)</f>
@@ -1412,7 +1474,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">IF(B8="AFP",ROUND(B21*INDEX(Parámetros!$B$18:$B$22,MATCH(B9,Parámetros!$A$18:$A$22,0)),2),0)</f>
@@ -1421,7 +1483,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">IF(B8="AFP",ROUND(B21*INDEX(Parámetros!$C$18:$C$22,MATCH(B9,Parámetros!$A$18:$A$22,0)),2),0)</f>
@@ -1430,7 +1492,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="B27" s="8" t="n">
         <f aca="false">IF(B8="AFP",ROUND(B21*INDEX(Parámetros!$D$18:$D$22,MATCH(B9,Parámetros!$A$18:$A$22,0)),2),0)</f>
@@ -1439,7 +1501,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="B28" s="8" t="n">
         <f aca="false">B12</f>
@@ -1447,25 +1509,25 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="19" t="s">
-        <v>60</v>
-      </c>
-      <c r="B29" s="20" t="n">
+      <c r="A29" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="B29" s="19" t="n">
         <f aca="false">SUM(B24:B28)</f>
         <v>621.27</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B32" s="8" t="n">
         <f aca="false">ROUND(B21*Parámetros!B9,2)</f>
@@ -1473,17 +1535,17 @@
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="21" t="s">
-        <v>63</v>
-      </c>
-      <c r="B34" s="22" t="n">
+      <c r="A34" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="B34" s="21" t="n">
         <f aca="false">B21-B29</f>
         <v>2631.73</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="B35" s="8" t="n">
         <f aca="false">B21+B32</f>
@@ -1492,9 +1554,9 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="B36" s="23" t="n">
+        <v>71</v>
+      </c>
+      <c r="B36" s="22" t="n">
         <f aca="false">B34/B35</f>
         <v>0.7422167822504</v>
       </c>
@@ -1554,94 +1616,94 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>26</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="I5" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="N5" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="J5" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="N5" s="3" t="s">
-        <v>53</v>
-      </c>
       <c r="O5" s="3" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="P5" s="3" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="Q5" s="3" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="R5" s="3" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="S5" s="3" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="T5" s="3" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="U5" s="3" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="V5" s="3" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="W5" s="3" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="X5" s="3" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="Y5" s="3" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
-        <v>83</v>
+      <c r="A6" s="18" t="s">
+        <v>89</v>
       </c>
       <c r="B6" s="5" t="n">
         <v>2500</v>
@@ -1650,16 +1712,16 @@
         <v>30</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="F6" s="11"/>
-      <c r="G6" s="24" t="n">
+      <c r="G6" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="24" t="n">
+      <c r="H6" s="23" t="n">
         <v>0</v>
       </c>
       <c r="I6" s="5" t="n">
@@ -1705,7 +1767,7 @@
         <f aca="false">IF($B6="","",SUM(O6:R6)+I6)</f>
         <v>325</v>
       </c>
-      <c r="T6" s="20" t="n">
+      <c r="T6" s="19" t="n">
         <f aca="false">IF($B6="","",N6-S6)</f>
         <v>2175</v>
       </c>
@@ -1720,15 +1782,15 @@
         <f aca="false">IF(V6="","sin dato en la guía",IF(ROUND(T6-V6,2)=0,"Sí","NO"))</f>
         <v>Sí</v>
       </c>
-      <c r="X6" s="15"/>
+      <c r="X6" s="13"/>
       <c r="Y6" s="8" t="str">
         <f aca="false">IF(X6="","",ROUND(X6-T6,2))</f>
         <v/>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
-        <v>85</v>
+      <c r="A7" s="18" t="s">
+        <v>91</v>
       </c>
       <c r="B7" s="5" t="n">
         <v>1800</v>
@@ -1737,16 +1799,16 @@
         <v>27</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="F7" s="11"/>
-      <c r="G7" s="24" t="n">
+      <c r="G7" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="24" t="n">
+      <c r="H7" s="23" t="n">
         <v>0</v>
       </c>
       <c r="I7" s="5" t="n">
@@ -1792,7 +1854,7 @@
         <f aca="false">IF($B7="","",SUM(O7:R7)+I7)</f>
         <v>226.59</v>
       </c>
-      <c r="T7" s="20" t="n">
+      <c r="T7" s="19" t="n">
         <f aca="false">IF($B7="","",N7-S7)</f>
         <v>1516.41</v>
       </c>
@@ -1807,15 +1869,15 @@
         <f aca="false">IF(V7="","sin dato en la guía",IF(ROUND(T7-V7,2)=0,"Sí","NO"))</f>
         <v>Sí</v>
       </c>
-      <c r="X7" s="15"/>
+      <c r="X7" s="13"/>
       <c r="Y7" s="8" t="str">
         <f aca="false">IF(X7="","",ROUND(X7-T7,2))</f>
         <v/>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
-        <v>86</v>
+      <c r="A8" s="18" t="s">
+        <v>92</v>
       </c>
       <c r="B8" s="5" t="n">
         <v>3000</v>
@@ -1824,7 +1886,7 @@
         <v>30</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="E8" s="11" t="s">
         <v>26</v>
@@ -1832,10 +1894,10 @@
       <c r="F8" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="G8" s="24" t="n">
+      <c r="G8" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="H8" s="24" t="n">
+      <c r="H8" s="23" t="n">
         <v>4</v>
       </c>
       <c r="I8" s="5" t="n">
@@ -1881,7 +1943,7 @@
         <f aca="false">IF($B8="","",SUM(O8:R8)+I8)</f>
         <v>621.27</v>
       </c>
-      <c r="T8" s="20" t="n">
+      <c r="T8" s="19" t="n">
         <f aca="false">IF($B8="","",N8-S8)</f>
         <v>2631.73</v>
       </c>
@@ -1896,15 +1958,15 @@
         <f aca="false">IF(V8="","sin dato en la guía",IF(ROUND(T8-V8,2)=0,"Sí","NO"))</f>
         <v>Sí</v>
       </c>
-      <c r="X8" s="15"/>
+      <c r="X8" s="13"/>
       <c r="Y8" s="8" t="str">
         <f aca="false">IF(X8="","",ROUND(X8-T8,2))</f>
         <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
-        <v>87</v>
+      <c r="A9" s="18" t="s">
+        <v>93</v>
       </c>
       <c r="B9" s="5" t="n">
         <v>4200</v>
@@ -1913,7 +1975,7 @@
         <v>24</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="E9" s="11" t="s">
         <v>26</v>
@@ -1921,10 +1983,10 @@
       <c r="F9" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="G9" s="24" t="n">
+      <c r="G9" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="H9" s="24" t="n">
+      <c r="H9" s="23" t="n">
         <v>2</v>
       </c>
       <c r="I9" s="5" t="n">
@@ -1970,7 +2032,7 @@
         <f aca="false">IF($B9="","",SUM(O9:R9)+I9)</f>
         <v>562.83</v>
       </c>
-      <c r="T9" s="20" t="n">
+      <c r="T9" s="19" t="n">
         <f aca="false">IF($B9="","",N9-S9)</f>
         <v>3011.17</v>
       </c>
@@ -1983,24 +2045,24 @@
         <f aca="false">IF(V9="","sin dato en la guía",IF(ROUND(T9-V9,2)=0,"Sí","NO"))</f>
         <v>sin dato en la guía</v>
       </c>
-      <c r="X9" s="15"/>
+      <c r="X9" s="13"/>
       <c r="Y9" s="8" t="str">
         <f aca="false">IF(X9="","",ROUND(X9-T9,2))</f>
         <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="19" t="s">
-        <v>88</v>
-      </c>
-      <c r="B10" s="15"/>
-      <c r="C10" s="16"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="15"/>
+      <c r="A10" s="18" t="s">
+        <v>94</v>
+      </c>
+      <c r="B10" s="13"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="13"/>
       <c r="J10" s="8" t="str">
         <f aca="false">IF($B10="","",ROUND(B10/Parámetros!$B$12*C10,2))</f>
         <v/>
@@ -2041,7 +2103,7 @@
         <f aca="false">IF($B10="","",SUM(O10:R10)+I10)</f>
         <v/>
       </c>
-      <c r="T10" s="20" t="str">
+      <c r="T10" s="19" t="str">
         <f aca="false">IF($B10="","",N10-S10)</f>
         <v/>
       </c>
@@ -2054,15 +2116,15 @@
         <f aca="false">IF(V10="","sin dato en la guía",IF(ROUND(T10-V10,2)=0,"Sí","NO"))</f>
         <v>sin dato en la guía</v>
       </c>
-      <c r="X10" s="15"/>
+      <c r="X10" s="13"/>
       <c r="Y10" s="8" t="str">
         <f aca="false">IF(X10="","",ROUND(X10-T10,2))</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="14" t="s">
-        <v>89</v>
+      <c r="A12" s="12" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -2093,43 +2155,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="25" t="s">
-        <v>49</v>
+      <c r="A5" s="24" t="s">
+        <v>55</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E5" s="8" t="n">
         <f aca="false">Casos!J8</f>
@@ -2137,17 +2199,17 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="25" t="s">
-        <v>50</v>
+      <c r="A6" s="24" t="s">
+        <v>56</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="E6" s="8" t="n">
         <f aca="false">Casos!K8</f>
@@ -2155,17 +2217,17 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25" t="s">
-        <v>103</v>
+      <c r="A7" s="24" t="s">
+        <v>109</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="E7" s="8" t="n">
         <f aca="false">Boleta!B16</f>
@@ -2173,17 +2235,17 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25" t="s">
-        <v>42</v>
+      <c r="A8" s="24" t="s">
+        <v>48</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="E8" s="8" t="n">
         <f aca="false">Casos!L8</f>
@@ -2191,17 +2253,17 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="25" t="s">
-        <v>43</v>
+      <c r="A9" s="24" t="s">
+        <v>49</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="E9" s="8" t="n">
         <f aca="false">Casos!M8</f>
@@ -2209,17 +2271,17 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="25" t="s">
-        <v>53</v>
+      <c r="A10" s="24" t="s">
+        <v>59</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="E10" s="8" t="n">
         <f aca="false">Casos!N8</f>
@@ -2227,17 +2289,17 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="25" t="s">
-        <v>55</v>
+      <c r="A11" s="24" t="s">
+        <v>61</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="E11" s="8" t="n">
         <f aca="false">Casos!O8</f>
@@ -2245,17 +2307,17 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="25" t="s">
-        <v>56</v>
+      <c r="A12" s="24" t="s">
+        <v>62</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="E12" s="8" t="n">
         <f aca="false">Casos!P8</f>
@@ -2263,17 +2325,17 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="25" t="s">
-        <v>57</v>
+      <c r="A13" s="24" t="s">
+        <v>63</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="E13" s="8" t="n">
         <f aca="false">Casos!Q8</f>
@@ -2281,17 +2343,17 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="25" t="s">
-        <v>58</v>
+      <c r="A14" s="24" t="s">
+        <v>64</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="E14" s="8" t="n">
         <f aca="false">Casos!R8</f>
@@ -2299,17 +2361,17 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="25" t="s">
-        <v>59</v>
+      <c r="A15" s="24" t="s">
+        <v>65</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="E15" s="8" t="n">
         <f aca="false">Casos!I8</f>
@@ -2317,17 +2379,17 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="25" t="s">
-        <v>60</v>
+      <c r="A16" s="24" t="s">
+        <v>66</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="E16" s="8" t="n">
         <f aca="false">Casos!S8</f>
@@ -2335,17 +2397,17 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="25" t="s">
-        <v>77</v>
+      <c r="A17" s="24" t="s">
+        <v>83</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="E17" s="8" t="n">
         <f aca="false">Casos!T8</f>
@@ -2353,17 +2415,17 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="25" t="s">
-        <v>78</v>
+      <c r="A18" s="24" t="s">
+        <v>84</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="E18" s="8" t="n">
         <f aca="false">Casos!U8</f>
@@ -2371,17 +2433,17 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="25" t="s">
-        <v>140</v>
+      <c r="A19" s="24" t="s">
+        <v>146</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="E19" s="8"/>
     </row>

</xml_diff>

<commit_message>
test: documentar 13 pruebas aprobadas y validar app contra Excel al centavo
</commit_message>
<xml_diff>
--- a/Semana 09/Boleta_Pago.xlsx
+++ b/Semana 09/Boleta_Pago.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parámetros" sheetId="1" r:id="Rd2bb131babfc446e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Boleta" sheetId="2" r:id="R9d10f2752fb04fbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos" sheetId="3" r:id="R41cd861c5156484c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Explicación" sheetId="4" r:id="Rbe0227ec9d114551"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parámetros" sheetId="1" r:id="Rc3a47730886e4300"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Boleta" sheetId="2" r:id="R7104b3556c95466d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos" sheetId="3" r:id="Raeb083b3ae624080"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Explicación" sheetId="4" r:id="Ra4ee94b955174031"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -293,9 +293,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Ejemplo numérico (caso 3)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Resultado en Excel (S/)</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">La parte del sueldo que realmente se ganó en el mes, según los días que se trabajó.</x:t>
@@ -601,7 +598,7 @@
     <x:xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <x:xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="35">
+  <x:cellXfs count="38">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -716,6 +713,17 @@
     </x:xf>
     <x:xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <x:alignment horizontal="general" vertical="top" wrapText="1" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="0" applyProtection="0">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
     </x:xf>
     <x:xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
@@ -1378,7 +1386,7 @@
       <x:c r="B15" s="3" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="D15" s="32" t="str">
+      <x:c r="D15" s="35" t="str">
         <x:v>Fórmula usada en Excel</x:v>
       </x:c>
     </x:row>
@@ -1390,7 +1398,7 @@
         <x:f aca="0">B5/Parámetros!B12/Parámetros!B13</x:f>
         <x:v>12.5</x:v>
       </x:c>
-      <x:c r="D16" s="34" t="str">
+      <x:c r="D16" s="37" t="str">
         <x:v>=B5/Parámetros!B12/Parámetros!B13</x:v>
       </x:c>
     </x:row>
@@ -1402,7 +1410,7 @@
         <x:f aca="0">ROUND(B5/Parámetros!B12*B6,2)</x:f>
         <x:v>3000</x:v>
       </x:c>
-      <x:c r="D17" s="34" t="str">
+      <x:c r="D17" s="37" t="str">
         <x:v>=ROUND(B5/Parámetros!B12*B6,2)</x:v>
       </x:c>
     </x:row>
@@ -1414,7 +1422,7 @@
         <x:f aca="0">IF(B7="Sí",ROUND(Parámetros!B7,2),0)</x:f>
         <x:v>123</x:v>
       </x:c>
-      <x:c r="D18" s="34" t="str">
+      <x:c r="D18" s="37" t="str">
         <x:v>=IF(B7="Sí",ROUND(Parámetros!B7,2),0)</x:v>
       </x:c>
     </x:row>
@@ -1426,7 +1434,7 @@
         <x:f aca="0">ROUND(B16*(1+Parámetros!B10)*B10,2)</x:f>
         <x:v>62.5</x:v>
       </x:c>
-      <x:c r="D19" s="34" t="str">
+      <x:c r="D19" s="37" t="str">
         <x:v>=ROUND(B16*(1+Parámetros!B10)*B10,2)</x:v>
       </x:c>
     </x:row>
@@ -1438,7 +1446,7 @@
         <x:f aca="0">ROUND(B16*(1+Parámetros!B11)*B11,2)</x:f>
         <x:v>67.5</x:v>
       </x:c>
-      <x:c r="D20" s="34" t="str">
+      <x:c r="D20" s="37" t="str">
         <x:v>=ROUND(B16*(1+Parámetros!B11)*B11,2)</x:v>
       </x:c>
     </x:row>
@@ -1450,12 +1458,12 @@
         <x:f aca="0">SUM(B17:B20)</x:f>
         <x:v>3253</x:v>
       </x:c>
-      <x:c r="D21" s="34" t="str">
+      <x:c r="D21" s="37" t="str">
         <x:v>=SUM(B17:B20)</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
-      <x:c r="D22" s="33"/>
+      <x:c r="D22" s="36"/>
     </x:row>
     <x:row r="23" ht="15" hidden="0">
       <x:c r="A23" s="3" t="s">
@@ -1464,7 +1472,7 @@
       <x:c r="B23" s="3" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="D23" s="33"/>
+      <x:c r="D23" s="36"/>
     </x:row>
     <x:row r="24" ht="34" hidden="0" customHeight="1">
       <x:c r="A24" s="4" t="s">
@@ -1474,7 +1482,7 @@
         <x:f aca="0">IF(B8="ONP",ROUND(B21*Parámetros!B8,2),0)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="D24" s="34" t="str">
+      <x:c r="D24" s="37" t="str">
         <x:v>=IF(B8="ONP",ROUND(B21*Parámetros!B8,2),0)</x:v>
       </x:c>
     </x:row>
@@ -1486,7 +1494,7 @@
         <x:f aca="0">IF(B8="AFP",ROUND(B21*INDEX(Parámetros!$B$18:$B$22,MATCH(B9,Parámetros!$A$18:$A$22,0)),2),0)</x:f>
         <x:v>325.3</x:v>
       </x:c>
-      <x:c r="D25" s="34" t="str">
+      <x:c r="D25" s="37" t="str">
         <x:v>=IF(B8="AFP",ROUND(B21*INDEX(Parámetros!$B$18:$B$22,MATCH(B9,Parámetros!$A$18:$A$22,0)),2),0)</x:v>
       </x:c>
     </x:row>
@@ -1498,7 +1506,7 @@
         <x:f aca="0">IF(B8="AFP",ROUND(B21*INDEX(Parámetros!$C$18:$C$22,MATCH(B9,Parámetros!$A$18:$A$22,0)),2),0)</x:f>
         <x:v>52.05</x:v>
       </x:c>
-      <x:c r="D26" s="34" t="str">
+      <x:c r="D26" s="37" t="str">
         <x:v>=IF(B8="AFP",ROUND(B21*INDEX(Parámetros!$C$18:$C$22,MATCH(B9,Parámetros!$A$18:$A$22,0)),2),0)</x:v>
       </x:c>
     </x:row>
@@ -1510,7 +1518,7 @@
         <x:f aca="0">IF(B8="AFP",ROUND(B21*INDEX(Parámetros!$D$18:$D$22,MATCH(B9,Parámetros!$A$18:$A$22,0)),2),0)</x:f>
         <x:v>43.92</x:v>
       </x:c>
-      <x:c r="D27" s="34" t="str">
+      <x:c r="D27" s="37" t="str">
         <x:v>=IF(B8="AFP",ROUND(B21*INDEX(Parámetros!$D$18:$D$22,MATCH(B9,Parámetros!$A$18:$A$22,0)),2),0)</x:v>
       </x:c>
     </x:row>
@@ -1522,7 +1530,7 @@
         <x:f aca="0">B12</x:f>
         <x:v>200</x:v>
       </x:c>
-      <x:c r="D28" s="34" t="str">
+      <x:c r="D28" s="37" t="str">
         <x:v>=B12</x:v>
       </x:c>
     </x:row>
@@ -1534,12 +1542,12 @@
         <x:f aca="0">SUM(B24:B28)</x:f>
         <x:v>621.27</x:v>
       </x:c>
-      <x:c r="D29" s="34" t="str">
+      <x:c r="D29" s="37" t="str">
         <x:v>=SUM(B24:B28)</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
-      <x:c r="D30" s="33"/>
+      <x:c r="D30" s="36"/>
     </x:row>
     <x:row r="31" ht="15" hidden="0">
       <x:c r="A31" s="3" t="s">
@@ -1548,7 +1556,7 @@
       <x:c r="B31" s="3" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="D31" s="33"/>
+      <x:c r="D31" s="36"/>
     </x:row>
     <x:row r="32" ht="34" hidden="0" customHeight="1">
       <x:c r="A32" s="4" t="s">
@@ -1558,12 +1566,12 @@
         <x:f aca="0">ROUND(B21*Parámetros!B9,2)</x:f>
         <x:v>292.77</x:v>
       </x:c>
-      <x:c r="D32" s="34" t="str">
+      <x:c r="D32" s="37" t="str">
         <x:v>=ROUND(B21*Parámetros!B9,2)</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
-      <x:c r="D33" s="33"/>
+      <x:c r="D33" s="36"/>
     </x:row>
     <x:row r="34" ht="34" hidden="0" customHeight="1">
       <x:c r="A34" s="20" t="s">
@@ -1573,7 +1581,7 @@
         <x:f aca="0">B21-B29</x:f>
         <x:v>2631.73</x:v>
       </x:c>
-      <x:c r="D34" s="34" t="str">
+      <x:c r="D34" s="37" t="str">
         <x:v>=B21-B29</x:v>
       </x:c>
     </x:row>
@@ -1585,7 +1593,7 @@
         <x:f aca="0">B21+B32</x:f>
         <x:v>3545.77</x:v>
       </x:c>
-      <x:c r="D35" s="34" t="str">
+      <x:c r="D35" s="37" t="str">
         <x:v>=B21+B32</x:v>
       </x:c>
     </x:row>
@@ -1597,13 +1605,13 @@
         <x:f aca="0">B34/B35</x:f>
         <x:v>0.7422167822503998</x:v>
       </x:c>
-      <x:c r="D36" s="34" t="str">
+      <x:c r="D36" s="37" t="str">
         <x:v>=B34/B35</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="28" customHeight="1">
       <x:c r="A38" t="str">
-        <x:v>Adelantos: máximo dos decimales. Los casos propios se completan después.</x:v>
+        <x:v>Para comparar con la app, ingresa adelantos al centavo. Casos propios pendientes.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1820,9 +1828,12 @@
         <x:f aca="0">IF(V6="","sin dato en la guía",IF(ROUND(T6-V6,2)=0,"Sí","NO"))</x:f>
         <x:v>Sí</x:v>
       </x:c>
-      <x:c r="X6" s="13"/>
-      <x:c r="Y6" s="8" t="str">
+      <x:c r="X6" s="13" t="n">
+        <x:v>2175</x:v>
+      </x:c>
+      <x:c r="Y6" s="8" t="n">
         <x:f aca="0">IF(X6="","",ROUND(X6-T6,2))</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0">
@@ -1906,9 +1917,12 @@
         <x:f aca="0">IF(V7="","sin dato en la guía",IF(ROUND(T7-V7,2)=0,"Sí","NO"))</x:f>
         <x:v>Sí</x:v>
       </x:c>
-      <x:c r="X7" s="13"/>
-      <x:c r="Y7" s="8" t="str">
+      <x:c r="X7" s="13" t="n">
+        <x:v>1516.41</x:v>
+      </x:c>
+      <x:c r="Y7" s="8" t="n">
         <x:f aca="0">IF(X7="","",ROUND(X7-T7,2))</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0">
@@ -1994,9 +2008,12 @@
         <x:f aca="0">IF(V8="","sin dato en la guía",IF(ROUND(T8-V8,2)=0,"Sí","NO"))</x:f>
         <x:v>Sí</x:v>
       </x:c>
-      <x:c r="X8" s="13"/>
-      <x:c r="Y8" s="8" t="str">
+      <x:c r="X8" s="13" t="n">
+        <x:v>2631.73</x:v>
+      </x:c>
+      <x:c r="Y8" s="8" t="n">
         <x:f aca="0">IF(X8="","",ROUND(X8-T8,2))</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0">
@@ -2080,9 +2097,12 @@
         <x:f aca="0">IF(V9="","sin dato en la guía",IF(ROUND(T9-V9,2)=0,"Sí","NO"))</x:f>
         <x:v>sin dato en la guía</x:v>
       </x:c>
-      <x:c r="X9" s="13"/>
-      <x:c r="Y9" s="8" t="str">
+      <x:c r="X9" s="13" t="n">
+        <x:v>3011.17</x:v>
+      </x:c>
+      <x:c r="Y9" s="8" t="n">
         <x:f aca="0">IF(X9="","",ROUND(X9-T9,2))</x:f>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0">
@@ -2148,7 +2168,21 @@
         <x:v>87</x:v>
       </x:c>
     </x:row>
+    <x:row r="14" ht="28" customHeight="1">
+      <x:c r="A14" t="str">
+        <x:v>Control cruzado ejecutado el 28/10/2026. Netos comprobados en el simulador iPhone 16 Pro, iOS 18.5. Diferencias en Y6:Y9: cero al centavo.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="28" customHeight="1">
+      <x:c r="A15" t="str">
+        <x:v>Evidencias y procedencia: evidencias/casos-swift.json, evidencias/simulador.log y PRUEBAS.md. El caso propio permanece pendiente.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A14:Y14"/>
+    <x:mergeCell ref="A15:Y15"/>
+  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
@@ -2187,8 +2221,8 @@
       <x:c r="D4" s="3" t="s">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="E4" s="3" t="s">
-        <x:v>94</x:v>
+      <x:c r="E4" s="3" t="str">
+        <x:v>Resultado (S/ o %)</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="43.5" hidden="0" customHeight="1">
@@ -2196,13 +2230,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="B5" s="6" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="C5" s="6" t="s">
+      <x:c r="D5" s="6" t="s">
         <x:v>96</x:v>
-      </x:c>
-      <x:c r="D5" s="6" t="s">
-        <x:v>97</x:v>
       </x:c>
       <x:c r="E5" s="8" t="n">
         <x:f aca="0">Casos!J8</x:f>
@@ -2214,13 +2248,13 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="B6" s="6" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="s">
         <x:v>98</x:v>
       </x:c>
-      <x:c r="C6" s="6" t="s">
+      <x:c r="D6" s="6" t="s">
         <x:v>99</x:v>
-      </x:c>
-      <x:c r="D6" s="6" t="s">
-        <x:v>100</x:v>
       </x:c>
       <x:c r="E6" s="8" t="n">
         <x:f aca="0">Casos!K8</x:f>
@@ -2229,16 +2263,16 @@
     </x:row>
     <x:row r="7" ht="43.5" hidden="0" customHeight="1">
       <x:c r="A7" s="24" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="s">
         <x:v>101</x:v>
       </x:c>
-      <x:c r="B7" s="6" t="s">
+      <x:c r="C7" s="6" t="s">
         <x:v>102</x:v>
       </x:c>
-      <x:c r="C7" s="6" t="s">
+      <x:c r="D7" s="6" t="s">
         <x:v>103</x:v>
-      </x:c>
-      <x:c r="D7" s="6" t="s">
-        <x:v>104</x:v>
       </x:c>
       <x:c r="E7" s="8" t="n">
         <x:f aca="0">Casos!B8/'Parámetros'!B12/'Parámetros'!B13</x:f>
@@ -2250,13 +2284,13 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="B8" s="6" t="s">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="s">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="C8" s="6" t="s">
+      <x:c r="D8" s="6" t="s">
         <x:v>106</x:v>
-      </x:c>
-      <x:c r="D8" s="6" t="s">
-        <x:v>107</x:v>
       </x:c>
       <x:c r="E8" s="8" t="n">
         <x:f aca="0">Casos!L8</x:f>
@@ -2268,13 +2302,13 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="B9" s="6" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="s">
         <x:v>108</x:v>
       </x:c>
-      <x:c r="C9" s="6" t="s">
+      <x:c r="D9" s="6" t="s">
         <x:v>109</x:v>
-      </x:c>
-      <x:c r="D9" s="6" t="s">
-        <x:v>110</x:v>
       </x:c>
       <x:c r="E9" s="8" t="n">
         <x:f aca="0">Casos!M8</x:f>
@@ -2286,13 +2320,13 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="B10" s="6" t="s">
+        <x:v>110</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="s">
         <x:v>111</x:v>
       </x:c>
-      <x:c r="C10" s="6" t="s">
+      <x:c r="D10" s="6" t="s">
         <x:v>112</x:v>
-      </x:c>
-      <x:c r="D10" s="6" t="s">
-        <x:v>113</x:v>
       </x:c>
       <x:c r="E10" s="8" t="n">
         <x:f aca="0">Casos!N8</x:f>
@@ -2304,13 +2338,13 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="B11" s="6" t="s">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="s">
         <x:v>114</x:v>
       </x:c>
-      <x:c r="C11" s="6" t="s">
+      <x:c r="D11" s="6" t="s">
         <x:v>115</x:v>
-      </x:c>
-      <x:c r="D11" s="6" t="s">
-        <x:v>116</x:v>
       </x:c>
       <x:c r="E11" s="8" t="n">
         <x:f aca="0">Casos!O8</x:f>
@@ -2322,13 +2356,13 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="B12" s="6" t="s">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="C12" s="6" t="s">
         <x:v>117</x:v>
       </x:c>
-      <x:c r="C12" s="6" t="s">
+      <x:c r="D12" s="6" t="s">
         <x:v>118</x:v>
-      </x:c>
-      <x:c r="D12" s="6" t="s">
-        <x:v>119</x:v>
       </x:c>
       <x:c r="E12" s="8" t="n">
         <x:f aca="0">Casos!P8</x:f>
@@ -2340,13 +2374,13 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="B13" s="6" t="s">
+        <x:v>119</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="s">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="C13" s="6" t="s">
+      <x:c r="D13" s="6" t="s">
         <x:v>121</x:v>
-      </x:c>
-      <x:c r="D13" s="6" t="s">
-        <x:v>122</x:v>
       </x:c>
       <x:c r="E13" s="8" t="n">
         <x:f aca="0">Casos!Q8</x:f>
@@ -2358,13 +2392,13 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="B14" s="6" t="s">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="C14" s="6" t="s">
         <x:v>123</x:v>
       </x:c>
-      <x:c r="C14" s="6" t="s">
+      <x:c r="D14" s="6" t="s">
         <x:v>124</x:v>
-      </x:c>
-      <x:c r="D14" s="6" t="s">
-        <x:v>125</x:v>
       </x:c>
       <x:c r="E14" s="8" t="n">
         <x:f aca="0">Casos!R8</x:f>
@@ -2376,13 +2410,13 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="B15" s="6" t="s">
+        <x:v>125</x:v>
+      </x:c>
+      <x:c r="C15" s="6" t="s">
         <x:v>126</x:v>
       </x:c>
-      <x:c r="C15" s="6" t="s">
+      <x:c r="D15" s="6" t="s">
         <x:v>127</x:v>
-      </x:c>
-      <x:c r="D15" s="6" t="s">
-        <x:v>128</x:v>
       </x:c>
       <x:c r="E15" s="8" t="n">
         <x:f aca="0">Casos!I8</x:f>
@@ -2394,13 +2428,13 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="B16" s="6" t="s">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="C16" s="6" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="C16" s="6" t="s">
+      <x:c r="D16" s="6" t="s">
         <x:v>130</x:v>
-      </x:c>
-      <x:c r="D16" s="6" t="s">
-        <x:v>131</x:v>
       </x:c>
       <x:c r="E16" s="8" t="n">
         <x:f aca="0">Casos!S8</x:f>
@@ -2412,13 +2446,13 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="B17" s="6" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="C17" s="6" t="s">
         <x:v>132</x:v>
       </x:c>
-      <x:c r="C17" s="6" t="s">
+      <x:c r="D17" s="6" t="s">
         <x:v>133</x:v>
-      </x:c>
-      <x:c r="D17" s="6" t="s">
-        <x:v>134</x:v>
       </x:c>
       <x:c r="E17" s="8" t="n">
         <x:f aca="0">Casos!T8</x:f>
@@ -2430,13 +2464,13 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="B18" s="6" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="C18" s="6" t="s">
         <x:v>135</x:v>
       </x:c>
-      <x:c r="C18" s="6" t="s">
+      <x:c r="D18" s="6" t="s">
         <x:v>136</x:v>
-      </x:c>
-      <x:c r="D18" s="6" t="s">
-        <x:v>137</x:v>
       </x:c>
       <x:c r="E18" s="8" t="n">
         <x:f aca="0">Casos!U8</x:f>
@@ -2445,18 +2479,54 @@
     </x:row>
     <x:row r="19" ht="43.5" hidden="0" customHeight="1">
       <x:c r="A19" s="24" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="B19" s="6" t="s">
         <x:v>138</x:v>
       </x:c>
-      <x:c r="B19" s="6" t="s">
+      <x:c r="C19" s="6" t="s">
         <x:v>139</x:v>
       </x:c>
-      <x:c r="C19" s="6" t="s">
+      <x:c r="D19" s="6" t="s">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="D19" s="6" t="s">
-        <x:v>141</x:v>
-      </x:c>
       <x:c r="E19" s="8"/>
+    </x:row>
+    <x:row r="20" ht="58" customHeight="1">
+      <x:c r="A20" s="24" t="str">
+        <x:v>Costo para el empleador</x:v>
+      </x:c>
+      <x:c r="B20" s="30" t="str">
+        <x:v>Lo que cuesta el trabajador en este modelo: remuneraciones más el aporte de salud.</x:v>
+      </x:c>
+      <x:c r="C20" s="30" t="str">
+        <x:v>Total remuneraciones + EsSalud.</x:v>
+      </x:c>
+      <x:c r="D20" s="30" t="str">
+        <x:v>3,253.00 + 292.77 = 3,545.77</x:v>
+      </x:c>
+      <x:c r="E20" s="31" t="n">
+        <x:f>Casos!N8+Casos!U8</x:f>
+        <x:v>3545.77</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="58" customHeight="1">
+      <x:c r="A21" s="24" t="str">
+        <x:v>Porcentaje del costo recibido</x:v>
+      </x:c>
+      <x:c r="B21" s="30" t="str">
+        <x:v>Parte del costo total que llega al trabajador como dinero neto.</x:v>
+      </x:c>
+      <x:c r="C21" s="30" t="str">
+        <x:v>Neto a pagar ÷ costo para el empleador × 100.</x:v>
+      </x:c>
+      <x:c r="D21" s="30" t="str">
+        <x:v>2,631.73 ÷ 3,545.77 × 100 = 74.22%</x:v>
+      </x:c>
+      <x:c r="E21" s="32" t="n">
+        <x:f>Casos!T8/E20</x:f>
+        <x:v>0.7422167822503998</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>